<commit_message>
Descreva aqui o que você alterou
</commit_message>
<xml_diff>
--- a/resumo_busca_ativa_consolidado.xlsx
+++ b/resumo_busca_ativa_consolidado.xlsx
@@ -119,12 +119,12 @@
     <t>PIRACANJUBA</t>
   </si>
   <si>
+    <t>RUBIATABA</t>
+  </si>
+  <si>
     <t>CIDADE OCIDENTAL</t>
   </si>
   <si>
-    <t>RUBIATABA</t>
-  </si>
-  <si>
     <t>PIRENOPOLIS</t>
   </si>
   <si>
@@ -161,12 +161,12 @@
     <t>MARA ROSA</t>
   </si>
   <si>
+    <t>GOIANAPOLIS</t>
+  </si>
+  <si>
     <t>COCALZINHO DE GOIAS</t>
   </si>
   <si>
-    <t>GOIANAPOLIS</t>
-  </si>
-  <si>
     <t>BURITI ALEGRE</t>
   </si>
   <si>
@@ -194,10 +194,10 @@
     <t>CRIXAS</t>
   </si>
   <si>
+    <t>NOVA CRIXAS</t>
+  </si>
+  <si>
     <t>PETROLINA DE GOIAS</t>
-  </si>
-  <si>
-    <t>NOVA CRIXAS</t>
   </si>
   <si>
     <t>CORUMBA DE GOIAS</t>
@@ -859,19 +859,19 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>19133</v>
+        <v>19106</v>
       </c>
       <c r="C2">
-        <v>2134</v>
+        <v>2341</v>
       </c>
       <c r="D2">
-        <v>1026</v>
+        <v>1015</v>
       </c>
       <c r="E2">
-        <v>15910</v>
+        <v>15676</v>
       </c>
       <c r="F2">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -879,19 +879,19 @@
         <v>7</v>
       </c>
       <c r="B3">
-        <v>16817</v>
+        <v>16796</v>
       </c>
       <c r="C3">
-        <v>1708</v>
+        <v>1979</v>
       </c>
       <c r="D3">
-        <v>1101</v>
+        <v>1169</v>
       </c>
       <c r="E3">
-        <v>13865</v>
+        <v>13454</v>
       </c>
       <c r="F3">
-        <v>114</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -899,19 +899,19 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>9446</v>
+        <v>9407</v>
       </c>
       <c r="C4">
-        <v>1135</v>
+        <v>1153</v>
       </c>
       <c r="D4">
-        <v>820</v>
+        <v>828</v>
       </c>
       <c r="E4">
-        <v>7259</v>
+        <v>7169</v>
       </c>
       <c r="F4">
-        <v>189</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>
@@ -949,16 +949,16 @@
         <v>10</v>
       </c>
       <c r="B2">
-        <v>9670</v>
+        <v>9660</v>
       </c>
       <c r="C2">
-        <v>875</v>
+        <v>975</v>
       </c>
       <c r="D2">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="E2">
-        <v>8336</v>
+        <v>8228</v>
       </c>
       <c r="F2">
         <v>14</v>
@@ -969,16 +969,16 @@
         <v>11</v>
       </c>
       <c r="B3">
-        <v>2381</v>
+        <v>2376</v>
       </c>
       <c r="C3">
-        <v>224</v>
+        <v>249</v>
       </c>
       <c r="D3">
-        <v>252</v>
+        <v>180</v>
       </c>
       <c r="E3">
-        <v>1815</v>
+        <v>1857</v>
       </c>
       <c r="F3">
         <v>83</v>
@@ -992,13 +992,13 @@
         <v>1735</v>
       </c>
       <c r="C4">
-        <v>139</v>
+        <v>202</v>
       </c>
       <c r="D4">
-        <v>187</v>
+        <v>155</v>
       </c>
       <c r="E4">
-        <v>1389</v>
+        <v>1358</v>
       </c>
       <c r="F4">
         <v>19</v>
@@ -1009,19 +1009,19 @@
         <v>13</v>
       </c>
       <c r="B5">
-        <v>1649</v>
+        <v>1644</v>
       </c>
       <c r="C5">
-        <v>179</v>
+        <v>223</v>
       </c>
       <c r="D5">
-        <v>221</v>
+        <v>303</v>
       </c>
       <c r="E5">
-        <v>1245</v>
+        <v>1091</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1029,16 +1029,16 @@
         <v>14</v>
       </c>
       <c r="B6">
-        <v>1500</v>
+        <v>1499</v>
       </c>
       <c r="C6">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="D6">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="E6">
-        <v>1037</v>
+        <v>1022</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -1049,16 +1049,16 @@
         <v>15</v>
       </c>
       <c r="B7">
-        <v>1280</v>
+        <v>1270</v>
       </c>
       <c r="C7">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="D7">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E7">
-        <v>956</v>
+        <v>945</v>
       </c>
       <c r="F7">
         <v>12</v>
@@ -1072,13 +1072,13 @@
         <v>1203</v>
       </c>
       <c r="C8">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D8">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="E8">
-        <v>1087</v>
+        <v>1061</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -1089,19 +1089,19 @@
         <v>17</v>
       </c>
       <c r="B9">
-        <v>1135</v>
+        <v>1132</v>
       </c>
       <c r="C9">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D9">
-        <v>219</v>
+        <v>239</v>
       </c>
       <c r="E9">
-        <v>763</v>
+        <v>713</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1109,16 +1109,16 @@
         <v>18</v>
       </c>
       <c r="B10">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="C10">
-        <v>163</v>
+        <v>202</v>
       </c>
       <c r="D10">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E10">
-        <v>800</v>
+        <v>762</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -1129,7 +1129,7 @@
         <v>19</v>
       </c>
       <c r="B11">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="C11">
         <v>70</v>
@@ -1138,7 +1138,7 @@
         <v>32</v>
       </c>
       <c r="E11">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -1152,16 +1152,16 @@
         <v>911</v>
       </c>
       <c r="C12">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E12">
-        <v>799</v>
+        <v>781</v>
       </c>
       <c r="F12">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1169,16 +1169,16 @@
         <v>21</v>
       </c>
       <c r="B13">
-        <v>843</v>
+        <v>840</v>
       </c>
       <c r="C13">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D13">
         <v>71</v>
       </c>
       <c r="E13">
-        <v>551</v>
+        <v>546</v>
       </c>
       <c r="F13">
         <v>101</v>
@@ -1192,13 +1192,13 @@
         <v>813</v>
       </c>
       <c r="C14">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D14">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="E14">
-        <v>773</v>
+        <v>750</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -1229,19 +1229,19 @@
         <v>24</v>
       </c>
       <c r="B16">
-        <v>790</v>
+        <v>783</v>
       </c>
       <c r="C16">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D16">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="E16">
-        <v>561</v>
+        <v>525</v>
       </c>
       <c r="F16">
-        <v>41</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1252,13 +1252,13 @@
         <v>729</v>
       </c>
       <c r="C17">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D17">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E17">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -1272,13 +1272,13 @@
         <v>695</v>
       </c>
       <c r="C18">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D18">
         <v>35</v>
       </c>
       <c r="E18">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="F18">
         <v>0</v>
@@ -1289,16 +1289,16 @@
         <v>27</v>
       </c>
       <c r="B19">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="C19">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D19">
-        <v>23</v>
+        <v>64</v>
       </c>
       <c r="E19">
-        <v>544</v>
+        <v>500</v>
       </c>
       <c r="F19">
         <v>0</v>
@@ -1312,13 +1312,13 @@
         <v>646</v>
       </c>
       <c r="C20">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D20">
         <v>35</v>
       </c>
       <c r="E20">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="F20">
         <v>0</v>
@@ -1329,16 +1329,16 @@
         <v>29</v>
       </c>
       <c r="B21">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="C21">
-        <v>145</v>
+        <v>182</v>
       </c>
       <c r="D21">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="E21">
-        <v>404</v>
+        <v>380</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -1349,16 +1349,16 @@
         <v>30</v>
       </c>
       <c r="B22">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="C22">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="D22">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="E22">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F22">
         <v>0</v>
@@ -1369,16 +1369,16 @@
         <v>31</v>
       </c>
       <c r="B23">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="C23">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D23">
         <v>71</v>
       </c>
       <c r="E23">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="F23">
         <v>17</v>
@@ -1389,16 +1389,16 @@
         <v>32</v>
       </c>
       <c r="B24">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C24">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D24">
         <v>14</v>
       </c>
       <c r="E24">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -1412,13 +1412,13 @@
         <v>495</v>
       </c>
       <c r="C25">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D25">
-        <v>8</v>
+        <v>41</v>
       </c>
       <c r="E25">
-        <v>411</v>
+        <v>375</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -1429,16 +1429,16 @@
         <v>34</v>
       </c>
       <c r="B26">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C26">
-        <v>100</v>
+        <v>53</v>
       </c>
       <c r="D26">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="E26">
-        <v>251</v>
+        <v>395</v>
       </c>
       <c r="F26">
         <v>0</v>
@@ -1449,16 +1449,16 @@
         <v>35</v>
       </c>
       <c r="B27">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="C27">
-        <v>49</v>
+        <v>95</v>
       </c>
       <c r="D27">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="E27">
-        <v>399</v>
+        <v>252</v>
       </c>
       <c r="F27">
         <v>0</v>
@@ -1472,13 +1472,13 @@
         <v>441</v>
       </c>
       <c r="C28">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D28">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="E28">
-        <v>356</v>
+        <v>366</v>
       </c>
       <c r="F28">
         <v>0</v>
@@ -1492,13 +1492,13 @@
         <v>406</v>
       </c>
       <c r="C29">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D29">
         <v>70</v>
       </c>
       <c r="E29">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="F29">
         <v>0</v>
@@ -1512,13 +1512,13 @@
         <v>402</v>
       </c>
       <c r="C30">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D30">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="E30">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="F30">
         <v>0</v>
@@ -1529,16 +1529,16 @@
         <v>39</v>
       </c>
       <c r="B31">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="C31">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D31">
-        <v>72</v>
+        <v>102</v>
       </c>
       <c r="E31">
-        <v>222</v>
+        <v>189</v>
       </c>
       <c r="F31">
         <v>0</v>
@@ -1549,16 +1549,16 @@
         <v>40</v>
       </c>
       <c r="B32">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C32">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="D32">
         <v>0</v>
       </c>
       <c r="E32">
-        <v>362</v>
+        <v>349</v>
       </c>
       <c r="F32">
         <v>0</v>
@@ -1572,13 +1572,13 @@
         <v>316</v>
       </c>
       <c r="C33">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D33">
         <v>0</v>
       </c>
       <c r="E33">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F33">
         <v>0</v>
@@ -1589,7 +1589,7 @@
         <v>42</v>
       </c>
       <c r="B34">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="C34">
         <v>50</v>
@@ -1598,7 +1598,7 @@
         <v>0</v>
       </c>
       <c r="E34">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="F34">
         <v>0</v>
@@ -1609,16 +1609,16 @@
         <v>43</v>
       </c>
       <c r="B35">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C35">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D35">
         <v>24</v>
       </c>
       <c r="E35">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F35">
         <v>0</v>
@@ -1629,16 +1629,16 @@
         <v>44</v>
       </c>
       <c r="B36">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C36">
-        <v>49</v>
+        <v>85</v>
       </c>
       <c r="D36">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="E36">
-        <v>196</v>
+        <v>137</v>
       </c>
       <c r="F36">
         <v>1</v>
@@ -1652,13 +1652,13 @@
         <v>238</v>
       </c>
       <c r="C37">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D37">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E37">
-        <v>146</v>
+        <v>194</v>
       </c>
       <c r="F37">
         <v>0</v>
@@ -1669,10 +1669,10 @@
         <v>46</v>
       </c>
       <c r="B38">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C38">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D38">
         <v>60</v>
@@ -1689,16 +1689,16 @@
         <v>47</v>
       </c>
       <c r="B39">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C39">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D39">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E39">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="F39">
         <v>0</v>
@@ -1709,16 +1709,16 @@
         <v>48</v>
       </c>
       <c r="B40">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C40">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="D40">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="E40">
-        <v>141</v>
+        <v>203</v>
       </c>
       <c r="F40">
         <v>0</v>
@@ -1729,16 +1729,16 @@
         <v>49</v>
       </c>
       <c r="B41">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C41">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="D41">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="E41">
-        <v>203</v>
+        <v>127</v>
       </c>
       <c r="F41">
         <v>0</v>
@@ -1758,7 +1758,7 @@
         <v>0</v>
       </c>
       <c r="E42">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F42">
         <v>0</v>
@@ -1769,16 +1769,16 @@
         <v>51</v>
       </c>
       <c r="B43">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C43">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="D43">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E43">
-        <v>166</v>
+        <v>133</v>
       </c>
       <c r="F43">
         <v>0</v>
@@ -1832,13 +1832,13 @@
         <v>182</v>
       </c>
       <c r="C46">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D46">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E46">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="F46">
         <v>3</v>
@@ -1872,13 +1872,13 @@
         <v>163</v>
       </c>
       <c r="C48">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D48">
         <v>0</v>
       </c>
       <c r="E48">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F48">
         <v>0</v>
@@ -1929,16 +1929,16 @@
         <v>59</v>
       </c>
       <c r="B51">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C51">
-        <v>62</v>
+        <v>17</v>
       </c>
       <c r="D51">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E51">
-        <v>66</v>
+        <v>111</v>
       </c>
       <c r="F51">
         <v>0</v>
@@ -1952,13 +1952,13 @@
         <v>150</v>
       </c>
       <c r="C52">
-        <v>15</v>
+        <v>65</v>
       </c>
       <c r="D52">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E52">
-        <v>128</v>
+        <v>85</v>
       </c>
       <c r="F52">
         <v>0</v>
@@ -2052,13 +2052,13 @@
         <v>128</v>
       </c>
       <c r="C57">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D57">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E57">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F57">
         <v>0</v>
@@ -2112,13 +2112,13 @@
         <v>124</v>
       </c>
       <c r="C60">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D60">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E60">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F60">
         <v>0</v>
@@ -2152,13 +2152,13 @@
         <v>118</v>
       </c>
       <c r="C62">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D62">
         <v>0</v>
       </c>
       <c r="E62">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F62">
         <v>0</v>
@@ -2192,13 +2192,13 @@
         <v>108</v>
       </c>
       <c r="C64">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D64">
         <v>0</v>
       </c>
       <c r="E64">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F64">
         <v>0</v>
@@ -2232,13 +2232,13 @@
         <v>107</v>
       </c>
       <c r="C66">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D66">
         <v>0</v>
       </c>
       <c r="E66">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F66">
         <v>0</v>
@@ -2252,10 +2252,10 @@
         <v>104</v>
       </c>
       <c r="C67">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D67">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E67">
         <v>60</v>
@@ -2412,13 +2412,13 @@
         <v>84</v>
       </c>
       <c r="C75">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D75">
         <v>0</v>
       </c>
       <c r="E75">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F75">
         <v>0</v>
@@ -2432,13 +2432,13 @@
         <v>81</v>
       </c>
       <c r="C76">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="D76">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E76">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="F76">
         <v>0</v>
@@ -2452,13 +2452,13 @@
         <v>81</v>
       </c>
       <c r="C77">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D77">
         <v>0</v>
       </c>
       <c r="E77">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F77">
         <v>0</v>
@@ -2472,13 +2472,13 @@
         <v>80</v>
       </c>
       <c r="C78">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D78">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E78">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F78">
         <v>0</v>
@@ -2632,13 +2632,13 @@
         <v>74</v>
       </c>
       <c r="C86">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D86">
         <v>0</v>
       </c>
       <c r="E86">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F86">
         <v>0</v>
@@ -2652,13 +2652,13 @@
         <v>72</v>
       </c>
       <c r="C87">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D87">
         <v>0</v>
       </c>
       <c r="E87">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F87">
         <v>0</v>
@@ -2712,13 +2712,13 @@
         <v>66</v>
       </c>
       <c r="C90">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D90">
         <v>0</v>
       </c>
       <c r="E90">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F90">
         <v>0</v>
@@ -2912,13 +2912,13 @@
         <v>58</v>
       </c>
       <c r="C100">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D100">
         <v>0</v>
       </c>
       <c r="E100">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F100">
         <v>0</v>
@@ -2995,10 +2995,10 @@
         <v>7</v>
       </c>
       <c r="D104">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E104">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F104">
         <v>1</v>
@@ -3072,13 +3072,13 @@
         <v>52</v>
       </c>
       <c r="C108">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D108">
         <v>0</v>
       </c>
       <c r="E108">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F108">
         <v>0</v>
@@ -3112,13 +3112,13 @@
         <v>52</v>
       </c>
       <c r="C110">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D110">
         <v>0</v>
       </c>
       <c r="E110">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F110">
         <v>0</v>
@@ -3138,10 +3138,10 @@
         <v>0</v>
       </c>
       <c r="E111">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="F111">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="112" spans="1:6">
@@ -3172,13 +3172,13 @@
         <v>48</v>
       </c>
       <c r="C113">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D113">
         <v>0</v>
       </c>
       <c r="E113">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F113">
         <v>0</v>
@@ -3209,10 +3209,10 @@
         <v>123</v>
       </c>
       <c r="B115">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C115">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D115">
         <v>0</v>
@@ -3412,13 +3412,13 @@
         <v>38</v>
       </c>
       <c r="C125">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D125">
         <v>0</v>
       </c>
       <c r="E125">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F125">
         <v>0</v>
@@ -3492,13 +3492,13 @@
         <v>36</v>
       </c>
       <c r="C129">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D129">
         <v>0</v>
       </c>
       <c r="E129">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F129">
         <v>0</v>
@@ -3532,13 +3532,13 @@
         <v>35</v>
       </c>
       <c r="C131">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D131">
         <v>0</v>
       </c>
       <c r="E131">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F131">
         <v>0</v>

</xml_diff>